<commit_message>
Update data TFL Riska & Ujang: LOA 19 ACC, 12 Tidak ACC, Word doc added
- LOA: 19 data ACC (8 asli + 11 pengganti/baru)
- LOA: 12 data Tidak ACC (11 Layak Huni, 1 tidak melanjutkan - Warsa)
- Lampegan: 6 data pengganti (highlight hijau)
- 5 orang LOA belum ada NIK/KK (Icah, Ekur, Carma, Ujang Jujun, Ujang Parman)
- Added Word (.docx) version
- All 3 formats: Excel, PDF, Word
</commit_message>
<xml_diff>
--- a/upload/Data_Riska_Ujang_TFL_IBUN.xlsx
+++ b/upload/Data_Riska_Ujang_TFL_IBUN.xlsx
@@ -5,6 +5,7 @@
   <sheets>
     <sheet name="Data Penerima" sheetId="1" r:id="rId1"/>
     <sheet name="Ringkasan" sheetId="2" r:id="rId2"/>
+    <sheet name="Tidak ACC - LOA" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -472,7 +473,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K2" t="str">
-        <v>Backlog 2 desil 2</v>
+        <v>ACC</v>
       </c>
       <c r="L2" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -511,7 +512,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K3" t="str">
-        <v>Tidak masuk backlog perumahan desil 4</v>
+        <v>ACC</v>
       </c>
       <c r="L3" t="str">
         <v>Tidak masuk backlog perumahan</v>
@@ -550,7 +551,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K4" t="str">
-        <v>Backlog 2 desil 4</v>
+        <v>ACC</v>
       </c>
       <c r="L4" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -589,7 +590,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K5" t="str">
-        <v>Backlog 1 desil 4</v>
+        <v>ACC</v>
       </c>
       <c r="L5" t="str">
         <v>Backlog 1 Desil 1-5</v>
@@ -628,7 +629,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K6" t="str">
-        <v>Backlog 2 desil 3</v>
+        <v>ACC</v>
       </c>
       <c r="L6" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -667,7 +668,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K7" t="str">
-        <v>Backlog 2 desil 2</v>
+        <v>ACC</v>
       </c>
       <c r="L7" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -706,7 +707,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K8" t="str">
-        <v>Backlog 1 desil 1</v>
+        <v>ACC</v>
       </c>
       <c r="L8" t="str">
         <v>Backlog 1 Desil 1-5</v>
@@ -745,7 +746,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K9" t="str">
-        <v>Backlog 2 desil 1</v>
+        <v>ACC</v>
       </c>
       <c r="L9" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -784,7 +785,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K10" t="str">
-        <v>Backlog 2 desil 2</v>
+        <v>ACC</v>
       </c>
       <c r="L10" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -822,7 +823,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K11" t="str">
-        <v>Tidak masuk backlog perumahan desil 1</v>
+        <v>ACC</v>
       </c>
       <c r="L11" t="str">
         <v>Tidak masuk backlog perumahan</v>
@@ -860,7 +861,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K12" t="str">
-        <v>Backlog 2 desil 6</v>
+        <v>ACC</v>
       </c>
       <c r="L12" t="str">
         <v>Backlog 2 Desil 6-10</v>
@@ -898,7 +899,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K13" t="str">
-        <v>Backlog 2 desil 4</v>
+        <v>ACC</v>
       </c>
       <c r="L13" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -936,7 +937,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K14" t="str">
-        <v>Tidak masuk backlog perumahan desil 6</v>
+        <v>ACC</v>
       </c>
       <c r="L14" t="str">
         <v>Tidak masuk backlog perumahan</v>
@@ -974,7 +975,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K15" t="str">
-        <v>Tidak masuk backlog perumahan desil 1</v>
+        <v>ACC</v>
       </c>
       <c r="L15" t="str">
         <v>Tidak masuk backlog perumahan</v>
@@ -1012,7 +1013,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K16" t="str">
-        <v>Backlog 2 desil 5</v>
+        <v>ACC</v>
       </c>
       <c r="L16" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1050,7 +1051,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K17" t="str">
-        <v>Backlog 2 desil 6 | Data Pengganti</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L17" t="str">
         <v>Backlog 2 Desil 6-10</v>
@@ -1088,7 +1089,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K18" t="str">
-        <v>Backlog 2 desil 1 | Data Pengganti</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L18" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1126,7 +1127,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K19" t="str">
-        <v>Backlog 2 desil 2 | Data Pengganti</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L19" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1164,7 +1165,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K20" t="str">
-        <v>Backlog 2 desil 2 | Data Pengganti</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L20" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1202,7 +1203,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K21" t="str">
-        <v>Backlog 2 desil 2 | Data Pengganti</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L21" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1240,7 +1241,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K22" t="str">
-        <v>Backlog 2 desil 1</v>
+        <v>ACC</v>
       </c>
       <c r="L22" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1278,7 +1279,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K23" t="str">
-        <v>Backlog 2 desil 1</v>
+        <v>ACC</v>
       </c>
       <c r="L23" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1316,7 +1317,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K24" t="str">
-        <v>Backlog 2 desil 3</v>
+        <v>ACC</v>
       </c>
       <c r="L24" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1354,7 +1355,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K25" t="str">
-        <v>Backlog 1 desil 4</v>
+        <v>ACC</v>
       </c>
       <c r="L25" t="str">
         <v>Backlog 1 Desil 1-5</v>
@@ -1392,7 +1393,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K26" t="str">
-        <v>Backlog 2 desil 2 | Data Pengganti</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L26" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1430,7 +1431,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K27" t="str">
-        <v>Backlog 2 desil 5</v>
+        <v>ACC</v>
       </c>
       <c r="L27" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1468,7 +1469,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K28" t="str">
-        <v>Tidak masuk backlog perumahan desil 3</v>
+        <v>ACC</v>
       </c>
       <c r="L28" t="str">
         <v>Tidak masuk backlog perumahan</v>
@@ -1506,7 +1507,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K29" t="str">
-        <v>Backlog 2 desil 2</v>
+        <v>ACC</v>
       </c>
       <c r="L29" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1544,7 +1545,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K30" t="str">
-        <v/>
+        <v>ACC</v>
       </c>
       <c r="L30" t="str">
         <v>-</v>
@@ -1582,7 +1583,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K31" t="str">
-        <v>Backlog 2 desil 3</v>
+        <v>ACC</v>
       </c>
       <c r="L31" t="str">
         <v>Backlog 2 Desil 1-5</v>
@@ -1620,7 +1621,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K32" t="str">
-        <v>-</v>
+        <v>ACC</v>
       </c>
       <c r="L32" t="str">
         <v>-</v>
@@ -1658,7 +1659,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K33" t="str">
-        <v>-</v>
+        <v>ACC</v>
       </c>
       <c r="L33" t="str">
         <v>-</v>
@@ -1696,7 +1697,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K34" t="str">
-        <v>-</v>
+        <v>ACC</v>
       </c>
       <c r="L34" t="str">
         <v>-</v>
@@ -1734,7 +1735,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K35" t="str">
-        <v>-</v>
+        <v>ACC</v>
       </c>
       <c r="L35" t="str">
         <v>-</v>
@@ -1772,7 +1773,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K36" t="str">
-        <v>Data Baru</v>
+        <v>ACC - Data Baru</v>
       </c>
       <c r="L36" t="str">
         <v>-</v>
@@ -1810,7 +1811,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K37" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L37" t="str">
         <v>-</v>
@@ -1848,7 +1849,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K38" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L38" t="str">
         <v>-</v>
@@ -1886,7 +1887,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K39" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L39" t="str">
         <v>-</v>
@@ -1924,7 +1925,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K40" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L40" t="str">
         <v>-</v>
@@ -1962,7 +1963,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K41" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L41" t="str">
         <v>-</v>
@@ -2000,7 +2001,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K42" t="str">
-        <v>-</v>
+        <v>ACC</v>
       </c>
       <c r="L42" t="str">
         <v>-</v>
@@ -2038,7 +2039,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K43" t="str">
-        <v>-</v>
+        <v>ACC</v>
       </c>
       <c r="L43" t="str">
         <v>-</v>
@@ -2076,7 +2077,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K44" t="str">
-        <v>-</v>
+        <v>ACC</v>
       </c>
       <c r="L44" t="str">
         <v>-</v>
@@ -2114,7 +2115,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K45" t="str">
-        <v>-</v>
+        <v>ACC</v>
       </c>
       <c r="L45" t="str">
         <v>-</v>
@@ -2152,7 +2153,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K46" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L46" t="str">
         <v>-</v>
@@ -2190,7 +2191,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K47" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L47" t="str">
         <v>-</v>
@@ -2228,7 +2229,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K48" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L48" t="str">
         <v>-</v>
@@ -2266,7 +2267,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K49" t="str">
-        <v>Data Pengganti</v>
+        <v>ACC</v>
       </c>
       <c r="L49" t="str">
         <v>-</v>
@@ -2304,7 +2305,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K50" t="str">
-        <v>Data Baru</v>
+        <v>ACC - Data Baru</v>
       </c>
       <c r="L50" t="str">
         <v>-</v>
@@ -2319,7 +2320,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -2398,7 +2399,7 @@
         <v>Laki-laki</v>
       </c>
       <c r="B10" t="str">
-        <v>51 orang</v>
+        <v>37 orang</v>
       </c>
     </row>
     <row r="11">
@@ -2406,12 +2407,355 @@
         <v>Perempuan</v>
       </c>
       <c r="B11" t="str">
-        <v>18 orang</v>
+        <v>12 orang</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>LOA - Tidak ACC</v>
+      </c>
+      <c r="B12" t="str">
+        <v>12 orang</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>LOA - ACC</v>
+      </c>
+      <c r="B13" t="str">
+        <v>19 orang</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Alasan Tidak ACC</v>
+      </c>
+      <c r="B14" t="str">
+        <v>11 Layak Huni, 1 Tidak Melanjutkan</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G13"/>
+  <cols>
+    <col min="1" max="1" width="5.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="5.83203125" customWidth="1"/>
+    <col min="4" max="4" width="20.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>NO</v>
+      </c>
+      <c r="B1" t="str">
+        <v>NAMA</v>
+      </c>
+      <c r="C1" t="str">
+        <v>L/P</v>
+      </c>
+      <c r="D1" t="str">
+        <v>NO KTP</v>
+      </c>
+      <c r="E1" t="str">
+        <v>NO KK</v>
+      </c>
+      <c r="F1" t="str">
+        <v>ALAMAT</v>
+      </c>
+      <c r="G1" t="str">
+        <v>ALASAN TIDAK ACC</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>EHA</v>
+      </c>
+      <c r="C2" t="str">
+        <v>P</v>
+      </c>
+      <c r="D2" t="str">
+        <v>3204355002550004</v>
+      </c>
+      <c r="E2" t="str">
+        <v>3204353009220015</v>
+      </c>
+      <c r="F2" t="str">
+        <v>KP. LOA RT 3 RW 10</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="str">
+        <v>LALAN</v>
+      </c>
+      <c r="C3" t="str">
+        <v>L</v>
+      </c>
+      <c r="D3" t="str">
+        <v>3204352905980001</v>
+      </c>
+      <c r="E3" t="str">
+        <v>3204351612210006</v>
+      </c>
+      <c r="F3" t="str">
+        <v>KP. CIDADAP RT 5 RW 5</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="str">
+        <v>WARSA</v>
+      </c>
+      <c r="C4" t="str">
+        <v>L</v>
+      </c>
+      <c r="D4" t="str">
+        <v>3204351002711001</v>
+      </c>
+      <c r="E4" t="str">
+        <v>3204351609140013</v>
+      </c>
+      <c r="F4" t="str">
+        <v>KP. BUKATANAH RT 2 RW 3</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Tidak ingin melanjutkan</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="str">
+        <v>U.ODIN</v>
+      </c>
+      <c r="C5" t="str">
+        <v>L</v>
+      </c>
+      <c r="D5" t="str">
+        <v>3204351108770005</v>
+      </c>
+      <c r="E5" t="str">
+        <v>3204351009120001</v>
+      </c>
+      <c r="F5" t="str">
+        <v>KP. MEKARSARI RT 3 RW 9</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ENDANG SARGA</v>
+      </c>
+      <c r="C6" t="str">
+        <v>L</v>
+      </c>
+      <c r="D6" t="str">
+        <v>3204350911550003</v>
+      </c>
+      <c r="E6" t="str">
+        <v>3204352903110009</v>
+      </c>
+      <c r="F6" t="str">
+        <v>KP. TIISDINGIN RT 2 RW 6</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="str">
+        <v>TOTO TARMALA</v>
+      </c>
+      <c r="C7" t="str">
+        <v>L</v>
+      </c>
+      <c r="D7" t="str">
+        <v>3204350101920031</v>
+      </c>
+      <c r="E7" t="str">
+        <v>3204351803050561</v>
+      </c>
+      <c r="F7" t="str">
+        <v>KP LOA RT 4 RW 2</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="str">
+        <v>UJANG TIMAN</v>
+      </c>
+      <c r="C8" t="str">
+        <v>L</v>
+      </c>
+      <c r="D8" t="str">
+        <v>3204351508760018</v>
+      </c>
+      <c r="E8" t="str">
+        <v>3204351211130013</v>
+      </c>
+      <c r="F8" t="str">
+        <v>KP LOA RT 4 RW 2</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="str">
+        <v>EMEH</v>
+      </c>
+      <c r="C9" t="str">
+        <v>P</v>
+      </c>
+      <c r="D9" t="str">
+        <v>3204354107590197</v>
+      </c>
+      <c r="E9" t="str">
+        <v>3204352210070031</v>
+      </c>
+      <c r="F9" t="str">
+        <v>MALINGPING RT 4 RW 8</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="str">
+        <v>TATAN RUSTANDI</v>
+      </c>
+      <c r="C10" t="str">
+        <v>L</v>
+      </c>
+      <c r="D10" t="str">
+        <v>3203151003900004</v>
+      </c>
+      <c r="E10" t="str">
+        <v>3204350304200001</v>
+      </c>
+      <c r="F10" t="str">
+        <v>KP LOA RT 4 RW 2</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="str">
+        <v>HADI</v>
+      </c>
+      <c r="C11" t="str">
+        <v>L</v>
+      </c>
+      <c r="D11" t="str">
+        <v>3204352502820008</v>
+      </c>
+      <c r="E11" t="str">
+        <v>3204351004070008</v>
+      </c>
+      <c r="F11" t="str">
+        <v>CIDADAP RT 5 RW 5</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ILPAN SETIA MULYA</v>
+      </c>
+      <c r="C12" t="str">
+        <v>L</v>
+      </c>
+      <c r="D12" t="str">
+        <v>3204332811900005</v>
+      </c>
+      <c r="E12" t="str">
+        <v>3204352506130041</v>
+      </c>
+      <c r="F12" t="str">
+        <v>KP. TIISDINGIN RT 1 RW 6</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" t="str">
+        <v>SAEPULOH</v>
+      </c>
+      <c r="C13" t="str">
+        <v>L</v>
+      </c>
+      <c r="D13" t="str">
+        <v>3204351406940003</v>
+      </c>
+      <c r="E13" t="str">
+        <v>3204352909220007</v>
+      </c>
+      <c r="F13" t="str">
+        <v>KP. LOA RT 3 RW 10</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Layak Huni</v>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update LOA: lengkapi NIK/KK semua 19 data ACC (Icah, Ekur, Carma Dedi, Ujang Jujun, Ujang Parman)
- ICAH: NIK 3204354107710061, KK 3204352304200006, Sempak RT 003 RW 005
- EKUR: NIK 3204354903820003, KK 3204351210230005, KP LOA RT 003 RW 010
- CARMA DEDI: NIK 3204351207600004, KK 3204350101060016, KP Cidadap RT 004 RW 005
- UJANG JUJUN: NIK 3204350204580001, KK 3204351803050591, KP Loa RT 003 RW 002
- UJANG PARMAN: NIK 3204351205570001, KK 3204351803051054, KP Lengo RT 004 RW 001
- Regenerate PDF
</commit_message>
<xml_diff>
--- a/upload/Data_Riska_Ujang_TFL_IBUN.xlsx
+++ b/upload/Data_Riska_Ujang_TFL_IBUN.xlsx
@@ -1621,7 +1621,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K32" t="str">
-        <v>ACC</v>
+        <v>ACC - Backlog 2 desil 5</v>
       </c>
       <c r="L32" t="str">
         <v>-</v>
@@ -1659,7 +1659,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K33" t="str">
-        <v>ACC</v>
+        <v>ACC - Backlog 2 desil 2</v>
       </c>
       <c r="L33" t="str">
         <v>-</v>
@@ -1697,7 +1697,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K34" t="str">
-        <v>ACC</v>
+        <v>ACC - Backlog 2 desil 1</v>
       </c>
       <c r="L34" t="str">
         <v>-</v>
@@ -1735,7 +1735,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K35" t="str">
-        <v>ACC</v>
+        <v>ACC - Backlog 2 desil 3</v>
       </c>
       <c r="L35" t="str">
         <v>-</v>
@@ -1811,7 +1811,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K37" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L37" t="str">
         <v>-</v>
@@ -1849,7 +1849,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K38" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L38" t="str">
         <v>-</v>
@@ -1887,7 +1887,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K39" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L39" t="str">
         <v>-</v>
@@ -1925,7 +1925,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K40" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L40" t="str">
         <v>-</v>
@@ -1942,13 +1942,13 @@
         <v>P</v>
       </c>
       <c r="D41" t="str">
-        <v>-</v>
+        <v>3204354107710061</v>
       </c>
       <c r="E41" t="str">
-        <v>-</v>
+        <v>3204352304200006</v>
       </c>
       <c r="F41" t="str">
-        <v>-</v>
+        <v>Sempak RT 003 RW 005</v>
       </c>
       <c r="G41" t="str">
         <v>LOA</v>
@@ -1963,7 +1963,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K41" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L41" t="str">
         <v>-</v>
@@ -2001,7 +2001,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K42" t="str">
-        <v>ACC</v>
+        <v>ACC - Backlog 2 desil 1</v>
       </c>
       <c r="L42" t="str">
         <v>-</v>
@@ -2039,7 +2039,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K43" t="str">
-        <v>ACC</v>
+        <v>ACC - Backlog 2 desil 1</v>
       </c>
       <c r="L43" t="str">
         <v>-</v>
@@ -2077,7 +2077,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K44" t="str">
-        <v>ACC</v>
+        <v>ACC - Backlog 2 desil 2</v>
       </c>
       <c r="L44" t="str">
         <v>-</v>
@@ -2115,7 +2115,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K45" t="str">
-        <v>ACC</v>
+        <v>ACC - Backlog 2 desil 2</v>
       </c>
       <c r="L45" t="str">
         <v>-</v>
@@ -2153,7 +2153,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K46" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L46" t="str">
         <v>-</v>
@@ -2170,13 +2170,13 @@
         <v>L</v>
       </c>
       <c r="D47" t="str">
-        <v>-</v>
+        <v>3204354903820003</v>
       </c>
       <c r="E47" t="str">
-        <v>-</v>
+        <v>3204351210230005</v>
       </c>
       <c r="F47" t="str">
-        <v>-</v>
+        <v>KP LOA RT 003 RW 010</v>
       </c>
       <c r="G47" t="str">
         <v>LOA</v>
@@ -2191,7 +2191,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K47" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L47" t="str">
         <v>-</v>
@@ -2202,19 +2202,19 @@
         <v>47</v>
       </c>
       <c r="B48" t="str">
-        <v>CARMA</v>
+        <v>CARMA DEDI</v>
       </c>
       <c r="C48" t="str">
         <v>L</v>
       </c>
       <c r="D48" t="str">
-        <v>-</v>
+        <v>3204351207600004</v>
       </c>
       <c r="E48" t="str">
-        <v>-</v>
+        <v>3204350101060016</v>
       </c>
       <c r="F48" t="str">
-        <v>-</v>
+        <v>KP CIDADAP RT 004 RW 005</v>
       </c>
       <c r="G48" t="str">
         <v>LOA</v>
@@ -2229,7 +2229,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K48" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L48" t="str">
         <v>-</v>
@@ -2246,13 +2246,13 @@
         <v>L</v>
       </c>
       <c r="D49" t="str">
-        <v>-</v>
+        <v>3204350204580001</v>
       </c>
       <c r="E49" t="str">
-        <v>-</v>
+        <v>3204351803050591</v>
       </c>
       <c r="F49" t="str">
-        <v>-</v>
+        <v>KP LOA RT 003 RW 002</v>
       </c>
       <c r="G49" t="str">
         <v>LOA</v>
@@ -2267,7 +2267,7 @@
         <v>JAWA BARAT</v>
       </c>
       <c r="K49" t="str">
-        <v>ACC</v>
+        <v>ACC - Data Pengganti</v>
       </c>
       <c r="L49" t="str">
         <v>-</v>
@@ -2284,13 +2284,13 @@
         <v>L</v>
       </c>
       <c r="D50" t="str">
-        <v>-</v>
+        <v>3204351205570001</v>
       </c>
       <c r="E50" t="str">
-        <v>-</v>
+        <v>3204351803051054</v>
       </c>
       <c r="F50" t="str">
-        <v>-</v>
+        <v>KP LENGO RT 004 RW 001</v>
       </c>
       <c r="G50" t="str">
         <v>LOA</v>
@@ -2444,15 +2444,6 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G13"/>
-  <cols>
-    <col min="1" max="1" width="5.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="5.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="28.83203125" customWidth="1"/>
-    <col min="7" max="7" width="28.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>